<commit_message>
Subindo atualizações de planilhas UC18 - UC35
</commit_message>
<xml_diff>
--- a/documentacao/Testes/Caso de Teste/UC18 - RELATÓRIO DE CAIXA.xlsx
+++ b/documentacao/Testes/Caso de Teste/UC18 - RELATÓRIO DE CAIXA.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="79">
   <si>
     <t xml:space="preserve">Caso de Teste</t>
   </si>
@@ -47,6 +47,9 @@
   </si>
   <si>
     <t xml:space="preserve">Observações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status de teste v2 (OK/NOK)</t>
   </si>
   <si>
     <t xml:space="preserve">CT01 - Gerar Relatório Diário</t>
@@ -350,7 +353,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -364,11 +367,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -494,8 +505,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.01"/>
@@ -532,294 +543,330 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="K1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="40.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="H2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="G4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="H4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="E5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="G5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="H5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="G6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="H6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="G7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="G8" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="H8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="G9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="E10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="G10" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="H10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="27.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="E11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="4" t="s">
+      <c r="G11" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="6" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>